<commit_message>
fix(training): mark mc16 Day1 AM + 1/13 as Specific (hard sessions)
These two Marathon sessions — 8km@4′30″+8km@3′45″ (mc16) and
3km+3*(1km@3′45″+1km) (1/13) — are hard, not base aerobic, so they
shouldn't inherit the cutback/day Fundamental rules. Marked them with the
Specific fill in the Excel, and generalized the race-fill override into
category_from_fill() so any category color set on a cell wins. Regenerate
plan.json; phase totals unchanged (1908 / 796.5 / 1160.6).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/running-log/2026-2nd-half.xlsx
+++ b/running-log/2026-2nd-half.xlsx
@@ -62,7 +62,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -134,6 +134,12 @@
     <fill>
       <patternFill/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6A9EE"/>
+        <bgColor rgb="FFF6A9EE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -154,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="6" fillId="13" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -276,6 +282,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -4279,7 +4291,7 @@
     </row>
     <row r="47">
       <c r="A47" s="29" t="inlineStr"/>
-      <c r="B47" s="17" t="inlineStr">
+      <c r="B47" s="43" t="inlineStr">
         <is>
           <t>8km@4′30″-4′40″ +8km@3′45″</t>
         </is>
@@ -4349,7 +4361,7 @@
           <t>7km Recovery +5*100m strides</t>
         </is>
       </c>
-      <c r="D50" s="41" t="inlineStr">
+      <c r="D50" s="44" t="inlineStr">
         <is>
           <t>3km wu +3*(1km@3′45″+1km@easy)</t>
         </is>

</xml_diff>

<commit_message>
chore(training): adjust aerobic phase mileage (mc17-27)
- Day 3 AM 非 cutback 统一 22km，加速课改 17+5km 格式
- Day 1 AM: 8/20 8/24 → 29km, 8/28 → 21+8km, 9/5 9/9 → 30km, 9/13 → 21+9km
</commit_message>
<xml_diff>
--- a/running-log/2026-2nd-half.xlsx
+++ b/running-log/2026-2nd-half.xlsx
@@ -1727,7 +1727,7 @@
       </c>
       <c r="D50" s="32" t="inlineStr">
         <is>
-          <t>23km Medium-Long Run @4′34″</t>
+          <t>22km Medium-Long Run @4′34″</t>
         </is>
       </c>
       <c r="E50" s="34" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="D53" s="32" t="inlineStr">
         <is>
-          <t>23km Medium-Long Run @4′30″</t>
+          <t>22km Medium-Long Run @4′30″</t>
         </is>
       </c>
       <c r="E53" s="34" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="D56" s="32" t="inlineStr">
         <is>
-          <t>17km@4′25″-4′30″ +6km@4′15″-4′20″</t>
+          <t>17km@4′25″-4′30″ +5km@4′15″-4′20″</t>
         </is>
       </c>
       <c r="E56" s="34" t="inlineStr">
@@ -1973,7 +1973,7 @@
       <c r="A62" s="29" t="inlineStr"/>
       <c r="B62" s="35" t="inlineStr">
         <is>
-          <t>28km Long Run @4′38″</t>
+          <t>29km Long Run @4′38″</t>
         </is>
       </c>
       <c r="C62" s="34" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="D62" s="32" t="inlineStr">
         <is>
-          <t>23km Medium-Long Run @4′30″</t>
+          <t>22km Medium-Long Run @4′30″</t>
         </is>
       </c>
       <c r="E62" s="34" t="inlineStr">
@@ -2037,7 +2037,7 @@
       <c r="A65" s="29" t="inlineStr"/>
       <c r="B65" s="35" t="inlineStr">
         <is>
-          <t>28km Long Run @4′34″</t>
+          <t>29km Long Run @4′34″</t>
         </is>
       </c>
       <c r="C65" s="34" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="D65" s="32" t="inlineStr">
         <is>
-          <t>23km Medium-Long Run @4′25″-4′30″</t>
+          <t>22km Medium-Long Run @4′25″-4′30″</t>
         </is>
       </c>
       <c r="E65" s="34" t="inlineStr">
@@ -2101,7 +2101,7 @@
       <c r="A68" s="29" t="inlineStr"/>
       <c r="B68" s="35" t="inlineStr">
         <is>
-          <t>20km@4′30″-4′35″ +8km@4′15″-4′25″</t>
+          <t>21km@4′30″-4′35″ +8km@4′15″-4′25″</t>
         </is>
       </c>
       <c r="C68" s="34" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="D68" s="32" t="inlineStr">
         <is>
-          <t>15km@4′22″-4′27″ +8km@4′12″-4′18″</t>
+          <t>17km@4′22″-4′27″ +5km@4′12″-4′18″</t>
         </is>
       </c>
       <c r="E68" s="34" t="inlineStr">
@@ -2229,7 +2229,7 @@
       <c r="A74" s="29" t="inlineStr"/>
       <c r="B74" s="35" t="inlineStr">
         <is>
-          <t>29km Long Run @4′35″-4′40″</t>
+          <t>30km Long Run @4′35″-4′40″</t>
         </is>
       </c>
       <c r="C74" s="34" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="D74" s="32" t="inlineStr">
         <is>
-          <t>24km Medium-Long Run @4′25″-4′30″</t>
+          <t>22km Medium-Long Run @4′25″-4′30″</t>
         </is>
       </c>
       <c r="E74" s="34" t="inlineStr">
@@ -2293,7 +2293,7 @@
       <c r="A77" s="29" t="inlineStr"/>
       <c r="B77" s="35" t="inlineStr">
         <is>
-          <t>29km Long Run @4′30″-4′35″</t>
+          <t>30km Long Run @4′30″-4′35″</t>
         </is>
       </c>
       <c r="C77" s="34" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D77" s="32" t="inlineStr">
         <is>
-          <t>24km Medium-Long Run @4′22″-4′27″</t>
+          <t>22km Medium-Long Run @4′22″-4′27″</t>
         </is>
       </c>
       <c r="E77" s="34" t="inlineStr">
@@ -2357,7 +2357,7 @@
       <c r="A80" s="29" t="inlineStr"/>
       <c r="B80" s="35" t="inlineStr">
         <is>
-          <t>19km@4′30″ +10km@4′15″-4′25″</t>
+          <t>21km@4′30″ +9km@4′15″-4′25″</t>
         </is>
       </c>
       <c r="C80" s="34" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="D80" s="32" t="inlineStr">
         <is>
-          <t>16km@4′20″-4′25″ +8km@4′10″-4′18″</t>
+          <t>17km@4′20″-4′25″ +5km@4′10″-4′18″</t>
         </is>
       </c>
       <c r="E80" s="34" t="inlineStr">

</xml_diff>